<commit_message>
Google Drive'dan otomatik Excel güncellemesi
</commit_message>
<xml_diff>
--- a/2026 YILI ÇAKABEY.xlsx
+++ b/2026 YILI ÇAKABEY.xlsx
@@ -22,12 +22,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="348">
+  <si>
+    <t>2026 YILI ÇAKABEY KÜLTÜR MERKEZİ</t>
+  </si>
   <si>
     <t xml:space="preserve">2026 YILI ÇAKABEY KÜLTÜR MERKEZİ </t>
   </si>
   <si>
-    <t>2026 YILI ÇAKABEY KÜLTÜR MERKEZİ</t>
+    <t>OCAK</t>
   </si>
   <si>
     <t xml:space="preserve">NİSAN </t>
@@ -55,43 +58,25 @@
     </r>
   </si>
   <si>
-    <t>OCAK</t>
+    <t xml:space="preserve"> 3 Ocak 2026 Cumartesi </t>
   </si>
   <si>
     <t xml:space="preserve">4 Nisan 2026 Cumartesi </t>
   </si>
   <si>
-    <t xml:space="preserve">2 Şubat 2026 Pazartesi </t>
+    <t>5 Ocak 2026 Pazartesi</t>
   </si>
   <si>
     <t xml:space="preserve">6 Nisan 2026 Pazartesi </t>
   </si>
   <si>
-    <t xml:space="preserve"> 3 Ocak 2026 Cumartesi </t>
-  </si>
-  <si>
-    <t>5 Ocak 2026 Pazartesi</t>
+    <t xml:space="preserve">10 Ocak 2026 Cumartesi </t>
   </si>
   <si>
     <t xml:space="preserve">11 Nisan 2026 Cumartesi </t>
   </si>
   <si>
     <t>Saygun Sanat Kırmızı Balık Müzikali 14.00 ve 16.00 2 seans dilekçe ve ödeme geldi.</t>
-  </si>
-  <si>
-    <t>Germiyan Köy Tiyatrosu Prova</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 Ocak 2026 Cumartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 Mart 2026 Pazartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 Şubat 2026 Cumartesi </t>
-  </si>
-  <si>
-    <t>CHP Eğitim 17.00-20.00</t>
   </si>
   <si>
     <t>Çeşme Belediyesi Türk Halk Müziği Korosu “ Çeşme’den Türkü Akıyor” 2026 Kış Konseri
@@ -100,52 +85,43 @@
 Çakabey Kültür Merkezi</t>
   </si>
   <si>
+    <t xml:space="preserve">2 Mart 2026 Pazartesi </t>
+  </si>
+  <si>
+    <t>Germiyan Köy Tiyatrosu Prova</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Esnaf ve Sanatkarlar odası toplantısı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Şubat 2026 Pazartesi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 Ocak 2026 Pazartesi </t>
+  </si>
+  <si>
     <t xml:space="preserve">7 Mart 2026 Cumartesi </t>
   </si>
   <si>
+    <t>CHP Eğitim 17.00-20.00</t>
+  </si>
+  <si>
+    <t>İstiklal Marşı Kabulü Provası</t>
+  </si>
+  <si>
     <t>Disk Dev EmekliSen Serdar Şahinkaya söyleşisi 15.00-18.00</t>
   </si>
   <si>
-    <t>Ot Festivali ile ilgili toplantı 14.00</t>
-  </si>
-  <si>
     <t>13 Nisan 2026 Pazartesi</t>
   </si>
   <si>
-    <t>İstiklal Marşı Kabulü Provası</t>
-  </si>
-  <si>
-    <t>İzmir Kent Tiyatrosu İlknur Barjit Çatal Tel No:05547273157         *14.00 Clown Sirki                       *20.00 Hafifletici Sebepler</t>
-  </si>
-  <si>
-    <t>Atatürkçü Düşünce Derneği Olağan Genel Kurul Toplantısı Deniz Ahilik Tel no: 05323416330</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9 Şubat 2026 Pazartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">14 Şubat 2026 Cumartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Esnaf ve Sanatkarlar odası toplantısı</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 Ocak 2026 Pazartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">*Sözleşmeli Personel Yemin Töreni Provası11.00                      *CHP İlçe Eğitim 17.00 Betül Araz tel no: 05539119496    </t>
-  </si>
-  <si>
-    <t>CHP İlçe Eğitim Betül Araz tel no: 05539119496</t>
-  </si>
-  <si>
-    <t>Tarladan Sofraya Gıda Güvenliği İZBB 14.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> *İnsan Kaynakları Yemin töreni 14.00</t>
-  </si>
-  <si>
-    <t>Belediye TSM Konseri Tüm gün</t>
+    <t xml:space="preserve">17 Ocak 2026 Cumartesi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 Nisan 2026 Cumartesi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 Şubat 2026 Cumartesi </t>
   </si>
   <si>
     <t>*İstiklal Marşı Kabulü Provası 09.30-14.30                            *Müdahil yetişkin oyunu dilekçe geldi ödeme alındı.</t>
@@ -155,46 +131,49 @@
 *16.00'dan sonra Dünyada Bir Yerde Oyunu Çeşme kent konseyi Deniz Karaman tel no:5356820132 Dilekçe geldi ödendi.</t>
   </si>
   <si>
-    <t xml:space="preserve">18 Nisan 2026 Cumartesi </t>
+    <t>İZBB Rahim Ağzı Kanseri ile ilgili konferans 13.30-15.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dijital Tarım Toplantısı 15.00 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarım Müdürü Şerif Bey için ayrıldı. Kavun Çalıştayı </t>
+  </si>
+  <si>
+    <t>Çeşme Kent Enstitüsü Tiyatro Çalışması</t>
+  </si>
+  <si>
+    <t>Ot Festivali ile ilgili toplantı 14.00</t>
   </si>
   <si>
     <t xml:space="preserve">9 Mart 2026 Pazartesi </t>
   </si>
   <si>
+    <t>İstanbul PAYE Çocuk Tiyatrosu Halil Soner Özaytekin tel no: 053340803734 seans onaylandı. Ödeme alındı.</t>
+  </si>
+  <si>
+    <t>İzmir Kent Tiyatrosu İlknur Barjit Çatal Tel No:05547273157         *14.00 Clown Sirki                       *20.00 Hafifletici Sebepler</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> KENT ENS. TİYATRO DERSİ (PAZARTESİ YAPILAMADIĞI İÇİN)</t>
+  </si>
+  <si>
+    <t>Atatürkçü Düşünce Derneği Olağan Genel Kurul Toplantısı Deniz Ahilik Tel no: 05323416330</t>
+  </si>
+  <si>
+    <t>YARI YIL ETKİNLİKLERİ</t>
+  </si>
+  <si>
     <t xml:space="preserve">14 Mart 2026 Cumartesi </t>
   </si>
   <si>
+    <t xml:space="preserve">9 Şubat 2026 Pazartesi </t>
+  </si>
+  <si>
     <t>18 Mart Provası sabahtan İstiklal Marşı Kabulü Provası</t>
   </si>
   <si>
-    <t>İstiklal Marşı Kabulü Kaymakamlık Etkinliği</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17 Ocak 2026 Cumartesi </t>
-  </si>
-  <si>
-    <t>Gezgin Kültür Sanat Hologram Çocuk Festivali 13.00-17.00 Deniz Gökpınar Tel no: 05072859296 Dilekçe geldi ve Ödendi. Onaylandı.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16 Mart 2026 Pazartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">16 Şubat 2026 Pazartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> KENT ENS. TİYATRO DERSİ (PAZARTESİ YAPILAMADIĞI İÇİN)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21 Mart 2026 Cumartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">21 Şubat 2026 Cumartesi </t>
-  </si>
-  <si>
-    <t>RAMAZAN BAYRAMI</t>
-  </si>
-  <si>
-    <t>İZBB Rahim Ağzı Kanseri ile ilgili konferans 13.30-15.00</t>
+    <t xml:space="preserve">14 Şubat 2026 Cumartesi </t>
   </si>
   <si>
     <r>
@@ -214,92 +193,113 @@
     </r>
   </si>
   <si>
+    <t>İstiklal Marşı Kabulü Kaymakamlık Etkinliği</t>
+  </si>
+  <si>
     <t>Artiz Mektebi 20.00                             Tiyatro Tirad Ücretsiz Oyun   Vedat Mehmet Korkmaz 05052926998</t>
   </si>
   <si>
-    <t xml:space="preserve">Dijital Tarım Toplantısı 15.00 </t>
+    <t>Gezgin Kültür Sanat Hologram Çocuk Festivali 13.00-17.00 Deniz Gökpınar Tel no: 05072859296 Dilekçe geldi ve Ödendi. Onaylandı.</t>
+  </si>
+  <si>
+    <t>19 Ocak 2026 Pazartesi</t>
   </si>
   <si>
     <t xml:space="preserve">20 Nisan 2026 Pazartesi </t>
   </si>
   <si>
+    <t xml:space="preserve">*Sözleşmeli Personel Yemin Töreni Provası11.00                      *CHP İlçe Eğitim 17.00 Betül Araz tel no: 05539119496    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 Mart 2026 Pazartesi </t>
+  </si>
+  <si>
+    <t>CHP İlçe Eğitim Betül Araz tel no: 05539119496</t>
+  </si>
+  <si>
+    <t>Tarladan Sofraya Gıda Güvenliği İZBB 14.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 Ocak 2026 Cumartesi </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> *İnsan Kaynakları Yemin töreni 14.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25 Nisan 2026 Cumartesi </t>
+  </si>
+  <si>
+    <t>Belediye TSM Konseri Tüm gün</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 Mart 2026 Cumartesi </t>
+  </si>
+  <si>
+    <t>İZMİR AŞKINA PROVA SAATİ BELLİ OLDUĞUNDA BİLGİ VERİLECEK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27 Nisan 2026 Pazartesi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 Ocak 2026 Pazartesi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 Şubat 2026 Pazartesi </t>
+  </si>
+  <si>
+    <t>RAMAZAN BAYRAMI</t>
+  </si>
+  <si>
+    <t>31 Ocak 2026 Cumartesi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 Şubat 2026 Cumartesi </t>
+  </si>
+  <si>
+    <t>İZBB Aronya Yetiştiriciliği Eğitimi</t>
+  </si>
+  <si>
+    <t>"Sokratesin Savunması".          Ödeme Geldi. Deniz Karaman: +90 (535) 682 01 32 İPTAL</t>
+  </si>
+  <si>
+    <t>İZBB Hayal Kasabası Çocuk Tiyatrosu 14.00</t>
+  </si>
+  <si>
     <t>CHP İlçe Eğitim için onaylandı. Betül Araz Tel no: 05539119496</t>
   </si>
   <si>
-    <t xml:space="preserve">Tarım Müdürü Şerif Bey için ayrıldı. Kavun Çalıştayı </t>
-  </si>
-  <si>
     <t>Çeşme Şoförler ve Otomobilciler Esnaf Odası Olağan Genel Kurulu Seçimi Tel No: 05326361993</t>
   </si>
   <si>
-    <t>Çeşme Kent Enstitüsü Tiyatro Çalışması</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 Nisan 2026 Cumartesi </t>
-  </si>
-  <si>
     <t>Edebiyat Dostları Derneği "Lüküs Hayat" için Onaylanlandı. Dilekçe geldi.                     Serap Hanım: 05359751764</t>
   </si>
   <si>
-    <t>İstanbul PAYE Çocuk Tiyatrosu Halil Soner Özaytekin tel no: 053340803734 seans onaylandı. Ödeme alındı.</t>
-  </si>
-  <si>
-    <t>İZMİR AŞKINA PROVA SAATİ BELLİ OLDUĞUNDA BİLGİ VERİLECEK</t>
+    <t xml:space="preserve">23 Mart 2026 Pazartesi </t>
   </si>
   <si>
     <t xml:space="preserve">23 Şubat 2026 Pazartesi </t>
   </si>
   <si>
-    <t>YARI YIL ETKİNLİKLERİ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27 Nisan 2026 Pazartesi </t>
+    <t xml:space="preserve">28 Mart 2026 Cumartesi </t>
   </si>
   <si>
     <t>28 Şubat 2026 Cumartesi</t>
   </si>
   <si>
-    <t>"Sokratesin Savunması".          Ödeme Geldi. Deniz Karaman: +90 (535) 682 01 32 İPTAL</t>
-  </si>
-  <si>
-    <t>19 Ocak 2026 Pazartesi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23 Mart 2026 Pazartesi </t>
-  </si>
-  <si>
-    <t>Ot festivali gıda ve ot stant toplantıları için opsiyonlandı</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 Ocak 2026 Cumartesi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">28 Mart 2026 Cumartesi </t>
-  </si>
-  <si>
     <t>CHP İlçe Eğitim tüm gün</t>
   </si>
   <si>
-    <t xml:space="preserve">26 Ocak 2026 Pazartesi </t>
-  </si>
-  <si>
     <t>Kaymakamlık 18 Mart Etkinliği Provası</t>
   </si>
   <si>
     <t xml:space="preserve">Kaymakamlık 18 Mart Etkinliği 8.30-13.00 arası </t>
-  </si>
-  <si>
-    <t>31 Ocak 2026 Cumartesi</t>
   </si>
   <si>
     <t>-Taşınmazın Pazarlıkla Satışı Adliye 11.00 
 -Çeşme Kaymakamlığı Himayesi Türk Halk Müziği Konseri 20.00</t>
   </si>
   <si>
-    <t>İZBB Aronya Yetiştiriciliği Eğitimi</t>
-  </si>
-  <si>
-    <t>İZBB Hayal Kasabası Çocuk Tiyatrosu 14.00</t>
+    <t>Ot festivali gıda ve ot stant toplantıları için opsiyonlandı</t>
   </si>
   <si>
     <t xml:space="preserve">30 Mart 2026 Pazartesi </t>
@@ -357,9 +357,6 @@
   </si>
   <si>
     <t xml:space="preserve">12 MAYIS 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 YILI  ÇAKABEY KÜLTÜR MERKEZİ </t>
   </si>
   <si>
     <t xml:space="preserve">13 MAYIS 2026 ÇARŞAMBA </t>
@@ -382,9 +379,6 @@
   <si>
     <t>Bilgiç Anaokulu Prova 
 10.30-15.30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HAZİRAN </t>
   </si>
   <si>
     <t xml:space="preserve">Bilgiç Anaokulu Prova 
@@ -428,9 +422,6 @@
   </si>
   <si>
     <t>Yabancı Dil Gecesi Provası Bilgiç Ortaokulu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 HAZİRAN 2026 PAZARTESİ </t>
   </si>
   <si>
     <r>
@@ -453,12 +444,42 @@
     <t>Yabancı Dil Gecesi Bilgiç Ortaokulu GÖSTERİ</t>
   </si>
   <si>
+    <t>BAYRAM</t>
+  </si>
+  <si>
+    <t>25 MAYIS 2026 PAZARTESİ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 MAYIS 2026 SALI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">27 MAYIS 2026 ÇARŞAMBA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 MAYIS 2026 PERŞEMBE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">29 MAYIS 2026 CUMA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 MAYIS 2026 CUMARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">31 MAYIS 2026 PAZAR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 YILI  ÇAKABEY KÜLTÜR MERKEZİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HAZİRAN </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 HAZİRAN 2026 PAZARTESİ </t>
+  </si>
+  <si>
     <t xml:space="preserve">2 HAZİRAN 2026 SALI </t>
   </si>
   <si>
-    <t>BAYRAM</t>
-  </si>
-  <si>
     <t xml:space="preserve">3 HAZİRAN 2026 ÇARŞAMBA </t>
   </si>
   <si>
@@ -468,28 +489,7 @@
     <t xml:space="preserve">5 HAZİRAN 2026 CUMA </t>
   </si>
   <si>
-    <t>25 MAYIS 2026 PAZARTESİ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26 MAYIS 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">27 MAYIS 2026 ÇARŞAMBA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">28 MAYIS 2026 PERŞEMBE </t>
-  </si>
-  <si>
     <t xml:space="preserve">6 HAZİRAN 2026 CUMARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">29 MAYIS 2026 CUMA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 MAYIS 2026 CUMARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">31 MAYIS 2026 PAZAR </t>
   </si>
   <si>
     <t>7 HAZİRAN 2026 PAZAR</t>
@@ -534,6 +534,9 @@
   <si>
     <t>Bilgiç İlkokulu 13.00 1. Sınıf Okuma Bayramı 18.00
 Çeşme Blediyespor Genel Kurul Toplantısı (bilgiçten sonra 1 saat)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEMMUZ </t>
   </si>
   <si>
     <t>İPTAL Lüküs Hayat Kabare onaylandı. Dilekçe ve ödeme geldi. İrem Özer tel no: 5359660071</t>
@@ -584,6 +587,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">4 TEMMUZ 2026 CUMARTESİ </t>
+  </si>
+  <si>
     <t>-SERTUR KOOPERATİF TOPLANTISI HALUK BEY 05336460236 
 15.00'a kadar
 - Kent Enstitüsü Prova</t>
@@ -598,6 +604,10 @@
     <t xml:space="preserve">15 HAZİRAN 2026 PAZARTESİ </t>
   </si>
   <si>
+    <t>Latin Katolik Kilisesi Ayin 
+18.30</t>
+  </si>
+  <si>
     <t xml:space="preserve">16 HAZİRAN 2026 SALI </t>
   </si>
   <si>
@@ -614,6 +624,12 @@
   </si>
   <si>
     <t xml:space="preserve">21 HAZİRAN 2026 PAZAR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 TEMMUZ 2026 PAZARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 TEMMUZ 2026 SALI </t>
   </si>
   <si>
     <t>Atatürk Lisesi tiyatro prova</t>
@@ -629,6 +645,9 @@
 sabahtan 21.00'a kadar</t>
   </si>
   <si>
+    <t xml:space="preserve">11 TEMMUZ 2026 CUMARTESİ </t>
+  </si>
+  <si>
     <t>-Namık Kemal Prova Okuma Bayramı 12.00'da bitecek                            -Thm Konseri</t>
   </si>
   <si>
@@ -636,59 +655,6 @@
   </si>
   <si>
     <t>Doğu Der Toplantı</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 HAZİRAN 2026 PAZARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">23 HAZİRAN 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 HAZİRAN 2026 ÇARŞAMBA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 HAZİRAN 2026 PERŞEMBE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">26 HAZİRAN 2026 CUMA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">27 HAZİRAN 2026 CUMARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">28 HAZİRAN 2026 PAZAR </t>
-  </si>
-  <si>
-    <t>Reyhan Cici Piyano Dinletisi
-Ödendi. Dilekçe geldi. Tel no:5320631925 12.00-20.00</t>
-  </si>
-  <si>
-    <t>MHP 15. Olağan Kongre Toplantısı</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29 HAZİRAN 2026 PAZARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 HAZİRAN 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEMMUZ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 TEMMUZ 2026 CUMARTESİ </t>
-  </si>
-  <si>
-    <t>Latin Katolik Kilisesi Ayin 
-18.30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 TEMMUZ 2026 PAZARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 TEMMUZ 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 TEMMUZ 2026 CUMARTESİ </t>
   </si>
   <si>
     <t>-Çoklu İklim Krizinin Gölgesinde Orman Yangınları
@@ -696,19 +662,53 @@
 -Belediye Meclisi 17.00'dan sonra</t>
   </si>
   <si>
+    <t xml:space="preserve">22 HAZİRAN 2026 PAZARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 HAZİRAN 2026 SALI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 HAZİRAN 2026 ÇARŞAMBA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">25 HAZİRAN 2026 PERŞEMBE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 HAZİRAN 2026 CUMA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">27 HAZİRAN 2026 CUMARTESİ </t>
+  </si>
+  <si>
     <t>Belediye meclisi 16.00'dan sonra</t>
   </si>
   <si>
+    <t xml:space="preserve">28 HAZİRAN 2026 PAZAR </t>
+  </si>
+  <si>
     <t>Saygın Sanat Arı Maya Müzikali.  2 seans 15.00-21.00</t>
   </si>
   <si>
     <t>Dem Parti Olağan Kurul 5445442823 Ali Güleser 19.00-22.00</t>
   </si>
   <si>
+    <t>Reyhan Cici Piyano Dinletisi
+Ödendi. Dilekçe geldi. Tel no:5320631925 12.00-20.00</t>
+  </si>
+  <si>
     <t xml:space="preserve">13 TEMMUZ 2026 PAZARTESİ </t>
   </si>
   <si>
+    <t>MHP 15. Olağan Kongre Toplantısı</t>
+  </si>
+  <si>
     <t xml:space="preserve">14 TEMMUZ 2026 SALI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">29 HAZİRAN 2026 PAZARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 HAZİRAN 2026 SALI </t>
   </si>
   <si>
     <t xml:space="preserve">18 TEMMUZ 2026 CUMARTESİ </t>
@@ -809,35 +809,125 @@
     <t xml:space="preserve">EYLÜL </t>
   </si>
   <si>
+    <t xml:space="preserve">EKİM </t>
+  </si>
+  <si>
     <t xml:space="preserve">1 EYLÜL 2026 SALI </t>
   </si>
   <si>
+    <t xml:space="preserve">1 EKİM  2026 PERŞEMBE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 EKİM 2026 CUMA </t>
+  </si>
+  <si>
+    <t>3 EKİM 2026 CUMARTESİ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 EKİM 2026 PAZAR </t>
+  </si>
+  <si>
     <t xml:space="preserve">5 EYLÜL 2026 CUMARTESİ </t>
+  </si>
+  <si>
+    <t>Yeni Parti Toplantı</t>
   </si>
   <si>
     <t>Tiyatro Kıvılcım Keloğlan Etkinliği ödendi
 Haydar Ali tel no: 5527151935</t>
   </si>
   <si>
+    <t>5 EKİM 2026 PAZARTESİ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 EKİM 2026 SALI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 EKİM 2026 ÇARŞAMBA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 EKİM 2026 PERŞEMBE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 EKİM 2026 CUMA </t>
+  </si>
+  <si>
     <t xml:space="preserve">7 EYLÜL 2026 PAZARTESİ </t>
   </si>
   <si>
+    <t xml:space="preserve">10 EKİM 2026 CUMARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 EKİM 2026 PAZAR </t>
+  </si>
+  <si>
     <t xml:space="preserve">8 EYLÜL 2026 SALI </t>
   </si>
   <si>
+    <t>Hafifletici Sebepler opsiyon</t>
+  </si>
+  <si>
+    <t>12 EKİM 2026 PAZARTESİ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 EKİM 2026 SALI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 EKİM 2026 ÇARŞAMBA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 EKİM 2026 PERŞEMBE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 EKİM 2026 CUMA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 EKİM 2026 CUMARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 EKİM 2026 PAZAR </t>
+  </si>
+  <si>
     <t xml:space="preserve">12 EYLÜL 2026 CUMARTESİ </t>
   </si>
   <si>
+    <t>KENT KONSEYİ OPSİYON (HER HAFTA ÇARŞAMBA 20.00 - 230.00 ARASI KULLANIM İÇİN DİLEKÇE YAZILACAK)</t>
+  </si>
+  <si>
     <t>Belediye Meclis 15.00 Tüm alan</t>
   </si>
   <si>
+    <t>İZMİR KENT TİYATROSU 05547273157</t>
+  </si>
+  <si>
     <t xml:space="preserve">14 EYLÜL 2026 PAZARTESİ </t>
   </si>
   <si>
+    <t>19 EKİM 2026 PAZARTESİ</t>
+  </si>
+  <si>
     <t xml:space="preserve">15 EYLÜL 2026 SALI </t>
   </si>
   <si>
+    <t xml:space="preserve">20 EKİM 2026 SALI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 EKİM 2026 ÇARŞAMBA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 EKİM 2026 PERŞEMBE </t>
+  </si>
+  <si>
     <t xml:space="preserve">19 EYLÜL 2026 CUMARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 EKİM 2026 CUMA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 EKİM 2026 CUMARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">25 EKİM 2026 PAZAR </t>
   </si>
   <si>
     <t xml:space="preserve">09:00-16:00 
@@ -845,14 +935,38 @@
 Müdürlüğü   ( İzmir Yurttaş Meclisi) </t>
   </si>
   <si>
+    <t>KENT KONSEYİ OPSİYON</t>
+  </si>
+  <si>
     <t xml:space="preserve">12:30-17:00
 İzmir Büyükşehir Belediyesi Sosyal Hizmetler Dairesi Başkanlığı Kentsel Adalet ve Eşitlik Şube
 Müdürlüğü   ( İzmir Yurttaş Meclisi) </t>
   </si>
   <si>
+    <t>KENT ENS. TİYATRO KURSİYER OYUNU "SEVGİLİ DOKTOR" AYSEL GÜZEL</t>
+  </si>
+  <si>
     <t>Çeşme Belediyespor Tekwando velileri toplantı 16.00-17.00</t>
   </si>
   <si>
+    <t xml:space="preserve">26 EKİM 2026 PAZARTESİ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">27 EKİM 2026 SALI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 EKİM 2026 ÇARŞAMBA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">29 EKİM 2026 PERŞEMBE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 EKİM 2026 CUMA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">31 EKİM 2026 CUMARTESİ </t>
+  </si>
+  <si>
     <t xml:space="preserve">21 EYLÜL 2026 PAZARTESİ </t>
   </si>
   <si>
@@ -860,9 +974,6 @@
   </si>
   <si>
     <t xml:space="preserve">26 EYLÜL 2026 CUMARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">EKİM </t>
   </si>
   <si>
     <t>Osman Uysal Konser Prova 18.00-22.00</t>
@@ -911,108 +1022,6 @@
   </si>
   <si>
     <t xml:space="preserve">29 EYLÜL 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 EKİM  2026 PERŞEMBE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 EKİM 2026 CUMA </t>
-  </si>
-  <si>
-    <t>3 EKİM 2026 CUMARTESİ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 EKİM 2026 PAZAR </t>
-  </si>
-  <si>
-    <t>Yeni Parti Toplantı</t>
-  </si>
-  <si>
-    <t>5 EKİM 2026 PAZARTESİ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 EKİM 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 EKİM 2026 ÇARŞAMBA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 EKİM 2026 PERŞEMBE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">9 EKİM 2026 CUMA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 EKİM 2026 CUMARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 EKİM 2026 PAZAR </t>
-  </si>
-  <si>
-    <t>Hafifletici Sebepler opsiyon</t>
-  </si>
-  <si>
-    <t>12 EKİM 2026 PAZARTESİ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 EKİM 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">14 EKİM 2026 ÇARŞAMBA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 EKİM 2026 PERŞEMBE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">16 EKİM 2026 CUMA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">17 EKİM 2026 CUMARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">18 EKİM 2026 PAZAR </t>
-  </si>
-  <si>
-    <t>İZMİR KENT TİYATROSU 05547273157</t>
-  </si>
-  <si>
-    <t>19 EKİM 2026 PAZARTESİ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 EKİM 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">21 EKİM 2026 ÇARŞAMBA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 EKİM 2026 PERŞEMBE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">23 EKİM 2026 CUMA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 EKİM 2026 CUMARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 EKİM 2026 PAZAR </t>
-  </si>
-  <si>
-    <t xml:space="preserve">26 EKİM 2026 PAZARTESİ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">27 EKİM 2026 SALI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">28 EKİM 2026 ÇARŞAMBA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">29 EKİM 2026 PERŞEMBE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 EKİM 2026 CUMA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">31 EKİM 2026 CUMARTESİ </t>
   </si>
   <si>
     <t xml:space="preserve">KASIM </t>
@@ -1244,6 +1253,7 @@
     </font>
     <font>
       <b/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -1256,14 +1266,13 @@
     </font>
     <font>
       <b/>
-      <sz val="15.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="15.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -1297,13 +1306,13 @@
     </font>
     <font>
       <b/>
+      <sz val="13.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="13.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -1324,14 +1333,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF6B26B"/>
-        <bgColor rgb="FFF6B26B"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFF9CB9C"/>
+        <bgColor rgb="FFF9CB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6B26B"/>
+        <bgColor rgb="FFF6B26B"/>
       </patternFill>
     </fill>
     <fill>
@@ -1342,26 +1357,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF9CB9C"/>
-        <bgColor rgb="FFF9CB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF93C47D"/>
         <bgColor rgb="FF93C47D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAD3"/>
-        <bgColor rgb="FFD9EAD3"/>
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFD9D9D9"/>
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -1433,112 +1442,115 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="1" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="8" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="8" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="4" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -1546,17 +1558,14 @@
     <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="9" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="9" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1574,62 +1583,65 @@
     <xf borderId="4" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="10" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="10" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="6" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="6" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="6" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="2" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="6" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" textRotation="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="14" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="14" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" textRotation="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="4" fillId="11" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="4" fillId="6" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" textRotation="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="15" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="15" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="11" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="4" fillId="11" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" textRotation="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="11" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
@@ -1904,212 +1916,212 @@
   </cols>
   <sheetData>
     <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="19">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="11">
         <v>46023.0</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="12">
         <v>46024.0</v>
       </c>
-      <c r="F3" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="19">
+      <c r="F3" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="11">
         <v>46026.0</v>
       </c>
     </row>
     <row r="4" ht="95.25" customHeight="1">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="12">
+        <v>46028.0</v>
+      </c>
+      <c r="C5" s="12">
+        <v>46029.0</v>
+      </c>
+      <c r="D5" s="12">
+        <v>46030.0</v>
+      </c>
+      <c r="E5" s="12">
+        <v>46031.0</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="16">
-        <v>46028.0</v>
-      </c>
-      <c r="C5" s="16">
-        <v>46029.0</v>
-      </c>
-      <c r="D5" s="16">
-        <v>46030.0</v>
-      </c>
-      <c r="E5" s="16">
-        <v>46031.0</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="19">
+      <c r="G5" s="11">
         <v>46033.0</v>
       </c>
     </row>
     <row r="6" ht="97.5" customHeight="1">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="26" t="s">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="9"/>
+      <c r="G6" s="21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" ht="18.0" customHeight="1">
+      <c r="A7" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="26" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" ht="18.0" customHeight="1">
-      <c r="A7" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="16">
+      <c r="B7" s="12">
         <v>46035.0</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="25">
         <v>46036.0</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="25">
         <v>46037.0</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="12">
         <v>46038.0</v>
       </c>
-      <c r="F7" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="33">
+      <c r="F7" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="28">
         <v>46040.0</v>
       </c>
     </row>
     <row r="8" ht="69.0" customHeight="1">
       <c r="A8" s="17" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="E8" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="34" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="12">
+        <v>46042.0</v>
+      </c>
+      <c r="C9" s="25">
+        <v>46043.0</v>
+      </c>
+      <c r="D9" s="25">
+        <v>46044.0</v>
+      </c>
+      <c r="E9" s="12">
+        <v>46045.0</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="11">
+        <v>46047.0</v>
+      </c>
+    </row>
+    <row r="10" ht="78.75" customHeight="1">
+      <c r="A10" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="27"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="36" t="s">
+      <c r="B11" s="12">
+        <v>46049.0</v>
+      </c>
+      <c r="C11" s="25">
+        <v>46050.0</v>
+      </c>
+      <c r="D11" s="25">
+        <v>46051.0</v>
+      </c>
+      <c r="E11" s="12">
+        <v>46052.0</v>
+      </c>
+      <c r="F11" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="G8" s="36" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="16">
-        <v>46042.0</v>
-      </c>
-      <c r="C9" s="28">
-        <v>46043.0</v>
-      </c>
-      <c r="D9" s="28">
-        <v>46044.0</v>
-      </c>
-      <c r="E9" s="16">
-        <v>46045.0</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="G9" s="19">
-        <v>46047.0</v>
-      </c>
-    </row>
-    <row r="10" ht="78.75" customHeight="1">
-      <c r="A10" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="F10" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" s="27"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="16">
-        <v>46049.0</v>
-      </c>
-      <c r="C11" s="28">
-        <v>46050.0</v>
-      </c>
-      <c r="D11" s="28">
-        <v>46051.0</v>
-      </c>
-      <c r="E11" s="16">
-        <v>46052.0</v>
-      </c>
-      <c r="F11" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="G11" s="8"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" ht="93.75" customHeight="1">
       <c r="A12" s="17"/>
       <c r="B12" s="17" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="C12" s="27"/>
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
       <c r="F12" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="G12" s="40"/>
+        <v>68</v>
+      </c>
+      <c r="G12" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2137,189 +2149,197 @@
   </cols>
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
-      <c r="A1" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="A1" s="58" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="25.5" customHeight="1">
-      <c r="A2" s="64" t="s">
-        <v>240</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="59" t="s">
+        <v>224</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="21" t="s">
-        <v>247</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>248</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>249</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>250</v>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="4" ht="84.0" customHeight="1">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
       <c r="D4" s="27"/>
       <c r="E4" s="27"/>
-      <c r="F4" s="49" t="s">
-        <v>251</v>
+      <c r="F4" s="60" t="s">
+        <v>231</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
-        <v>252</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>253</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>254</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>255</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>256</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>257</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>258</v>
+      <c r="A5" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="6" ht="93.75" customHeight="1">
       <c r="A6" s="27"/>
       <c r="B6" s="27"/>
-      <c r="C6" s="65" t="s">
-        <v>259</v>
+      <c r="C6" s="63" t="s">
+        <v>242</v>
       </c>
       <c r="D6" s="27"/>
       <c r="E6" s="27"/>
-      <c r="F6" s="66" t="s">
-        <v>259</v>
+      <c r="F6" s="60" t="s">
+        <v>242</v>
       </c>
       <c r="G6" s="27"/>
-      <c r="L6" s="67"/>
+      <c r="L6" s="65"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
-        <v>260</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>261</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>262</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>263</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>264</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>265</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>266</v>
+      <c r="A7" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="8" ht="97.5" customHeight="1">
       <c r="A8" s="27"/>
       <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
+      <c r="C8" s="67" t="s">
+        <v>251</v>
+      </c>
       <c r="D8" s="27"/>
       <c r="E8" s="27"/>
       <c r="F8" s="68" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="G8" s="27"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>268</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>269</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>270</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>271</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>272</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>274</v>
+      <c r="A9" s="19" t="s">
+        <v>255</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>259</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="10" ht="100.5" customHeight="1">
       <c r="A10" s="27"/>
       <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
+      <c r="C10" s="60" t="s">
+        <v>265</v>
+      </c>
       <c r="D10" s="27"/>
       <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
+      <c r="F10" s="67" t="s">
+        <v>267</v>
+      </c>
       <c r="G10" s="27"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>275</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>276</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>277</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>278</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>279</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>280</v>
-      </c>
-      <c r="G11" s="8"/>
+      <c r="A11" s="19" t="s">
+        <v>269</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>271</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>272</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" ht="94.5" customHeight="1">
       <c r="A12" s="27"/>
       <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
+      <c r="C12" s="60" t="s">
+        <v>265</v>
+      </c>
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
       <c r="F12" s="27"/>
-      <c r="G12" s="8"/>
+      <c r="G12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2346,67 +2366,67 @@
   <sheetData>
     <row r="1" ht="33.75" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="25.5" customHeight="1">
       <c r="A2" s="42" t="s">
-        <v>281</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+        <v>284</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3" ht="18.75" customHeight="1">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="21" t="s">
-        <v>282</v>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="19" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="4" ht="87.75" customHeight="1">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
       <c r="G4" s="27"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
-        <v>283</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>284</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>285</v>
-      </c>
-      <c r="D5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>286</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>287</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>289</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>291</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="6" ht="98.25" customHeight="1">
@@ -2419,26 +2439,26 @@
       <c r="G6" s="27"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
-        <v>290</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>291</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>292</v>
-      </c>
-      <c r="D7" s="21" t="s">
+      <c r="A7" s="19" t="s">
         <v>293</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>294</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>295</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>296</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="8" ht="98.25" customHeight="1">
@@ -2451,26 +2471,26 @@
       <c r="G8" s="27"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>297</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>298</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>299</v>
-      </c>
-      <c r="D9" s="21" t="s">
+      <c r="A9" s="19" t="s">
         <v>300</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>301</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>302</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>303</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>304</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="10" ht="107.25" customHeight="1">
@@ -2483,26 +2503,26 @@
       <c r="G10" s="27"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>304</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>306</v>
-      </c>
-      <c r="D11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>307</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="B11" s="19" t="s">
         <v>308</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="D11" s="19" t="s">
         <v>310</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>311</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>312</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="12" ht="103.5" customHeight="1">
@@ -2512,29 +2532,29 @@
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
       <c r="F12" s="27"/>
-      <c r="G12" s="69" t="s">
-        <v>311</v>
+      <c r="G12" s="70" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="s">
-        <v>312</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="A13" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
     </row>
     <row r="14" ht="90.75" customHeight="1">
       <c r="A14" s="27"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2563,49 +2583,49 @@
   <sheetData>
     <row r="1" ht="35.25" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="21.75" customHeight="1">
-      <c r="A2" s="50" t="s">
-        <v>313</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="51" t="s">
+        <v>316</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3">
       <c r="A3" s="43"/>
-      <c r="B3" s="21" t="s">
-        <v>314</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>315</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>316</v>
-      </c>
-      <c r="E3" s="21" t="s">
+      <c r="B3" s="19" t="s">
         <v>317</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>318</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="D3" s="19" t="s">
         <v>319</v>
       </c>
+      <c r="E3" s="19" t="s">
+        <v>320</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>321</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="4" ht="91.5" customHeight="1">
-      <c r="A4" s="8"/>
+      <c r="A4" s="9"/>
       <c r="B4" s="27"/>
       <c r="C4" s="27"/>
       <c r="D4" s="27"/>
@@ -2614,26 +2634,26 @@
       <c r="G4" s="27"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
-        <v>320</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>321</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>322</v>
-      </c>
-      <c r="D5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>323</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>324</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>326</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>327</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="6" ht="99.0" customHeight="1">
@@ -2646,26 +2666,26 @@
       <c r="G6" s="27"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
-        <v>327</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>328</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>329</v>
-      </c>
-      <c r="D7" s="21" t="s">
+      <c r="A7" s="19" t="s">
         <v>330</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>331</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>332</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>333</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>334</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>335</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="8" ht="96.0" customHeight="1">
@@ -2678,26 +2698,26 @@
       <c r="G8" s="27"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>334</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>335</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>336</v>
-      </c>
-      <c r="D9" s="21" t="s">
+      <c r="A9" s="19" t="s">
         <v>337</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>338</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>339</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>340</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>341</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>342</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="10" ht="96.75" customHeight="1">
@@ -2710,30 +2730,30 @@
       <c r="G10" s="27"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>341</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>342</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>343</v>
-      </c>
-      <c r="D11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>344</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="B11" s="19" t="s">
+        <v>345</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>346</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>347</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" ht="90.0" customHeight="1">
       <c r="A12" s="27"/>
       <c r="B12" s="27"/>
       <c r="C12" s="27"/>
       <c r="D12" s="27"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2762,13 +2782,13 @@
   <sheetData>
     <row r="1" ht="63.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
@@ -2785,14 +2805,14 @@
       <c r="T1" s="6"/>
     </row>
     <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
@@ -2809,13 +2829,13 @@
       <c r="T2" s="6"/>
     </row>
     <row r="3">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="12">
+      <c r="A3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="18">
         <v>46054.0</v>
       </c>
       <c r="H3" s="6"/>
@@ -2833,12 +2853,12 @@
       <c r="T3" s="6"/>
     </row>
     <row r="4" ht="86.25" customHeight="1">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="13"/>
+      <c r="A4" s="16"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="20"/>
       <c r="G4" s="17"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
@@ -2855,25 +2875,25 @@
       <c r="T4" s="6"/>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="22">
+      <c r="A5" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="26">
         <v>46056.0</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="26">
         <v>46057.0</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="26">
         <v>46058.0</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="26">
         <v>46059.0</v>
       </c>
-      <c r="F5" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="12">
+      <c r="F5" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="18">
         <v>46061.0</v>
       </c>
       <c r="H5" s="6"/>
@@ -2892,17 +2912,17 @@
     </row>
     <row r="6" ht="93.75" customHeight="1">
       <c r="A6" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
+        <v>33</v>
+      </c>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
       <c r="F6" s="17" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -2919,25 +2939,25 @@
       <c r="T6" s="6"/>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="22">
+      <c r="A7" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="26">
         <v>46063.0</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="26">
         <v>46064.0</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="26">
         <v>46065.0</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="26">
         <v>46066.0</v>
       </c>
-      <c r="F7" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="12">
+      <c r="F7" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="18">
         <v>46068.0</v>
       </c>
       <c r="H7" s="6"/>
@@ -2955,22 +2975,22 @@
       <c r="T7" s="6"/>
     </row>
     <row r="8" ht="105.75" customHeight="1">
-      <c r="A8" s="11"/>
+      <c r="A8" s="16"/>
       <c r="B8" s="17" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="11"/>
-      <c r="G8" s="31" t="s">
-        <v>34</v>
+        <v>55</v>
+      </c>
+      <c r="F8" s="16"/>
+      <c r="G8" s="35" t="s">
+        <v>57</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
@@ -2987,25 +3007,25 @@
       <c r="T8" s="6"/>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="22">
+      <c r="A9" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="26">
         <v>46070.0</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="26">
         <v>46071.0</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="26">
         <v>46072.0</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="26">
         <v>46073.0</v>
       </c>
-      <c r="F9" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="12">
+      <c r="F9" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="18">
         <v>46075.0</v>
       </c>
       <c r="H9" s="6"/>
@@ -3024,17 +3044,17 @@
     </row>
     <row r="10" ht="89.25" customHeight="1">
       <c r="A10" s="17"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
       <c r="E10" s="17" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
@@ -3051,25 +3071,25 @@
       <c r="T10" s="6"/>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" s="22">
+      <c r="A11" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="26">
         <v>46077.0</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="26">
         <v>46078.0</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="26">
         <v>46079.0</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="26">
         <v>46080.0</v>
       </c>
-      <c r="F11" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="G11" s="11"/>
+      <c r="F11" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" s="16"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
@@ -3085,15 +3105,15 @@
       <c r="T11" s="6"/>
     </row>
     <row r="12" ht="98.25" customHeight="1">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
       <c r="D12" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
+        <v>80</v>
+      </c>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
@@ -24406,147 +24426,147 @@
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="23.25" customHeight="1">
       <c r="A2" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+        <v>4</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="19">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="11">
         <v>46082.0</v>
       </c>
     </row>
     <row r="4" ht="69.0" customHeight="1">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
       <c r="G4" s="17" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="16">
+      <c r="A5" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="12">
         <v>46084.0</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="12">
         <v>46085.0</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="12">
         <v>46086.0</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="12">
         <v>46087.0</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="11">
         <v>46089.0</v>
       </c>
     </row>
     <row r="6" ht="113.25" customHeight="1">
-      <c r="A6" s="8"/>
+      <c r="A6" s="9"/>
       <c r="B6" s="27" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" s="27"/>
       <c r="D6" s="17" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="F6" s="17"/>
-      <c r="G6" s="29"/>
+      <c r="G6" s="31"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="16">
+      <c r="A7" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="12">
         <v>46091.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="12">
         <v>46092.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="12">
         <v>46093.0</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="12">
         <v>46094.0</v>
       </c>
-      <c r="F7" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="19">
+      <c r="F7" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" s="11">
         <v>46096.0</v>
       </c>
     </row>
     <row r="8" ht="87.0" customHeight="1">
-      <c r="A8" s="8"/>
+      <c r="A8" s="9"/>
       <c r="B8" s="27" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" s="8"/>
+        <v>45</v>
+      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="G8" s="8"/>
+        <v>47</v>
+      </c>
+      <c r="G8" s="9"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="16">
+      <c r="A9" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="12">
         <v>46098.0</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="11">
         <v>46099.0</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="25">
         <v>46100.0</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="12">
         <v>46101.0</v>
       </c>
-      <c r="F9" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" s="19">
+      <c r="F9" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="11">
         <v>46103.0</v>
       </c>
     </row>
@@ -24554,74 +24574,74 @@
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
-      <c r="D10" s="35" t="s">
-        <v>49</v>
-      </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="D10" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
       <c r="G10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="B11" s="16">
+      <c r="A11" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="12">
         <v>46105.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="12">
         <v>46106.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="12">
         <v>46107.0</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="12">
         <v>46108.0</v>
       </c>
-      <c r="F11" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="19">
+      <c r="F11" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" s="11">
         <v>46110.0</v>
       </c>
     </row>
     <row r="12" ht="91.5" customHeight="1">
-      <c r="A12" s="8"/>
+      <c r="A12" s="9"/>
       <c r="B12" s="17" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
+        <v>79</v>
+      </c>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="12">
         <v>46112.0</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
     </row>
     <row r="14" ht="95.25" customHeight="1">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -24650,195 +24670,195 @@
   </cols>
   <sheetData>
     <row r="1" ht="33.75" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="A1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="21.0" customHeight="1">
-      <c r="A2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3" ht="17.25" customHeight="1">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="16">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="12">
         <v>46113.0</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="12">
         <v>46114.0</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="12">
         <v>46115.0</v>
       </c>
-      <c r="F3" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="19">
+      <c r="F3" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="11">
         <v>46117.0</v>
       </c>
     </row>
     <row r="4" ht="99.75" customHeight="1">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="17"/>
-      <c r="G4" s="8"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="16">
+      <c r="A5" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="12">
         <v>46119.0</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="12">
         <v>46120.0</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="12">
         <v>46121.0</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="12">
         <v>46122.0</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="11">
         <v>46124.0</v>
       </c>
     </row>
     <row r="6" ht="78.0" customHeight="1">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="25" t="s">
-        <v>17</v>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>20</v>
       </c>
       <c r="F6" s="17"/>
-      <c r="G6" s="23" t="s">
-        <v>20</v>
+      <c r="G6" s="22" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="7" ht="21.0" customHeight="1">
-      <c r="A7" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="16">
+      <c r="A7" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="12">
         <v>46126.0</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="25">
         <v>46127.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="12">
         <v>46128.0</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="12">
         <v>46129.0</v>
       </c>
-      <c r="F7" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="19">
+      <c r="F7" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="11">
         <v>46131.0</v>
       </c>
     </row>
     <row r="8" ht="80.25" customHeight="1">
       <c r="A8" s="30"/>
       <c r="B8" s="32"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="34" t="s">
+      <c r="C8" s="9"/>
+      <c r="D8" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="17"/>
+      <c r="G8" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="23" t="s">
-        <v>52</v>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="16">
+      <c r="A9" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="12">
         <v>46133.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="12">
         <v>46134.0</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="11">
         <v>46135.0</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="12">
         <v>46136.0</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" s="11">
+        <v>46138.0</v>
+      </c>
+    </row>
+    <row r="10" ht="92.25" customHeight="1">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="G9" s="19">
-        <v>46138.0</v>
-      </c>
-    </row>
-    <row r="10" ht="92.25" customHeight="1">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" s="16">
+      <c r="A11" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="12">
         <v>46140.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="12">
         <v>46141.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="12">
         <v>46142.0</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" ht="98.25" customHeight="1">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
       <c r="D12" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
     </row>
     <row r="13">
-      <c r="D13" s="38"/>
+      <c r="D13" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -24867,84 +24887,84 @@
   <sheetData>
     <row r="1" ht="37.5" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="42" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3" ht="18.75" customHeight="1">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="18" t="s">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="15" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="4" ht="94.5" customHeight="1">
-      <c r="A4" s="8"/>
+      <c r="A4" s="9"/>
       <c r="B4" s="43"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
       <c r="E4" s="44" t="s">
         <v>86</v>
       </c>
       <c r="F4" s="45"/>
-      <c r="G4" s="23" t="s">
+      <c r="G4" s="22" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="5" ht="20.25" customHeight="1">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="E5" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="15" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="6" ht="91.5" customHeight="1">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="23" t="s">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="D6" s="8"/>
+      <c r="D6" s="9"/>
       <c r="E6" s="46" t="s">
         <v>96</v>
       </c>
@@ -24954,139 +24974,139 @@
       <c r="G6" s="45"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="E7" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="F7" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="G7" s="15" t="s">
         <v>104</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="8" ht="97.5" customHeight="1">
       <c r="A8" s="17"/>
       <c r="B8" s="48" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="D8" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="D8" s="23" t="s">
+      <c r="E8" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" s="47" t="s">
         <v>109</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="G8" s="22" t="s">
         <v>110</v>
       </c>
-      <c r="F8" s="47" t="s">
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="G8" s="23" t="s">
+      <c r="B9" s="15" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="s">
+      <c r="C9" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="E9" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="F9" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="G9" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="F9" s="18" t="s">
+    </row>
+    <row r="10" ht="93.75" customHeight="1">
+      <c r="A10" s="22" t="s">
         <v>118</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" ht="93.75" customHeight="1">
-      <c r="A10" s="23" t="s">
-        <v>120</v>
       </c>
       <c r="B10" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="E10" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="F10" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="G10" s="50" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="B11" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="F10" s="51" t="s">
+      <c r="C11" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="D11" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="G10" s="51" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="G11" s="18" t="s">
-        <v>137</v>
+      <c r="E11" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="12" ht="109.5" customHeight="1">
-      <c r="A12" s="51" t="s">
-        <v>126</v>
-      </c>
-      <c r="B12" s="51" t="s">
-        <v>126</v>
-      </c>
-      <c r="C12" s="51" t="s">
-        <v>126</v>
-      </c>
-      <c r="D12" s="51" t="s">
-        <v>126</v>
-      </c>
-      <c r="E12" s="51" t="s">
-        <v>126</v>
-      </c>
-      <c r="F12" s="51" t="s">
-        <v>126</v>
-      </c>
-      <c r="G12" s="51" t="s">
-        <v>126</v>
+      <c r="A12" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="B12" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="E12" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="F12" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="G12" s="50" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -25116,51 +25136,51 @@
   <sheetData>
     <row r="1" ht="58.5" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="30.0" customHeight="1">
-      <c r="A2" s="50" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="51" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>128</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>129</v>
-      </c>
-      <c r="F3" s="18" t="s">
+      <c r="A3" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="D3" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="G3" s="15" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="4" ht="91.5" customHeight="1">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>139</v>
       </c>
       <c r="B4" s="17" t="s">
@@ -25173,126 +25193,126 @@
         <v>142</v>
       </c>
       <c r="E4" s="52" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F4" s="37" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G4" s="17"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="C5" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="D5" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="F5" s="15" t="s">
         <v>150</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="6" ht="183.75" customHeight="1">
       <c r="A6" s="53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C6" s="53" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>153</v>
-      </c>
-      <c r="E6" s="25" t="s">
         <v>154</v>
       </c>
+      <c r="E6" s="24" t="s">
+        <v>156</v>
+      </c>
       <c r="F6" s="54" t="s">
-        <v>155</v>
-      </c>
-      <c r="G6" s="23" t="s">
-        <v>156</v>
+        <v>157</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
-        <v>157</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>158</v>
-      </c>
-      <c r="C7" s="21" t="s">
+      <c r="A7" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="D7" s="21" t="s">
-        <v>160</v>
-      </c>
-      <c r="E7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>163</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="8" ht="101.25" customHeight="1">
       <c r="A8" s="49" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C8" s="49" t="s">
-        <v>166</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>168</v>
+        <v>171</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>174</v>
       </c>
       <c r="F8" s="49" t="s">
-        <v>169</v>
-      </c>
-      <c r="G8" s="23" t="s">
-        <v>170</v>
+        <v>175</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>171</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>173</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>177</v>
+      <c r="A9" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="10" ht="99.75" customHeight="1">
@@ -25301,25 +25321,25 @@
       <c r="C10" s="27"/>
       <c r="D10" s="27"/>
       <c r="E10" s="27"/>
-      <c r="F10" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>179</v>
+      <c r="F10" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>180</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>181</v>
-      </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="A11" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" ht="107.25" customHeight="1">
       <c r="A12" s="27"/>
@@ -25357,115 +25377,115 @@
   <sheetData>
     <row r="1" ht="33.75" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="24.0" customHeight="1">
-      <c r="A2" s="50" t="s">
-        <v>182</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="16">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="12">
         <v>46204.0</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="12">
         <v>46205.0</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="12">
         <v>46206.0</v>
       </c>
-      <c r="F3" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="G3" s="19">
+      <c r="F3" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="G3" s="11">
         <v>46208.0</v>
       </c>
     </row>
     <row r="4" ht="91.5" customHeight="1">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="27"/>
       <c r="D4" s="27"/>
       <c r="E4" s="27"/>
       <c r="F4" s="49" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="G4" s="17"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
-        <v>185</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="C5" s="16">
+      <c r="A5" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="C5" s="12">
         <v>46211.0</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="12">
         <v>46212.0</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F5" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="G5" s="19">
+      <c r="F5" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="G5" s="11">
         <v>46215.0</v>
       </c>
     </row>
     <row r="6" ht="92.25" customHeight="1">
       <c r="A6" s="55" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="B6" s="27"/>
       <c r="C6" s="27"/>
       <c r="D6" s="49" t="s">
+        <v>184</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>160</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="E6" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="F6" s="49" t="s">
-        <v>184</v>
-      </c>
-      <c r="G6" s="23" t="s">
+      <c r="B7" s="19" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="21" t="s">
-        <v>192</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>193</v>
-      </c>
-      <c r="C7" s="28">
+      <c r="C7" s="25">
         <v>46218.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="12">
         <v>46219.0</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="12">
         <v>46220.0</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="15" t="s">
         <v>194</v>
       </c>
       <c r="G7" s="56">
@@ -25479,30 +25499,30 @@
       <c r="D8" s="27"/>
       <c r="E8" s="27"/>
       <c r="F8" s="49" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="G8" s="27"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="12">
         <v>46225.0</v>
       </c>
       <c r="D9" s="57">
         <v>46226.0</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="11">
         <v>46229.0</v>
       </c>
     </row>
@@ -25520,32 +25540,32 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="12">
         <v>46232.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="12">
         <v>46233.0</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="E11" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" ht="90.75" customHeight="1">
       <c r="A12" s="27"/>
       <c r="B12" s="27"/>
       <c r="C12" s="27"/>
       <c r="D12" s="27"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -25574,70 +25594,70 @@
   <sheetData>
     <row r="1" ht="34.5" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="24.75" customHeight="1">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="51" t="s">
         <v>203</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="18" t="s">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="G3" s="19">
+      <c r="G3" s="11">
         <v>46236.0</v>
       </c>
     </row>
     <row r="4" ht="94.5" customHeight="1">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="49" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="G4" s="27"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="12">
         <v>46239.0</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="12">
         <v>46240.0</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="12">
         <v>46241.0</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="11">
         <v>46243.0</v>
       </c>
     </row>
@@ -25647,31 +25667,31 @@
       <c r="C6" s="27"/>
       <c r="D6" s="27"/>
       <c r="E6" s="27"/>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="22" t="s">
         <v>208</v>
       </c>
       <c r="G6" s="27"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="12">
         <v>46246.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="12">
         <v>46247.0</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="12">
         <v>46248.0</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="G7" s="19">
+      <c r="G7" s="11">
         <v>46250.0</v>
       </c>
     </row>
@@ -25682,30 +25702,30 @@
       <c r="D8" s="27"/>
       <c r="E8" s="27"/>
       <c r="F8" s="49" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="G8" s="27"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="12">
         <v>46253.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="12">
         <v>46254.0</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="12">
         <v>46255.0</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="11">
         <v>46257.0</v>
       </c>
     </row>
@@ -25714,38 +25734,38 @@
       <c r="B10" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="C10" s="40"/>
+      <c r="C10" s="38"/>
       <c r="D10" s="49" t="s">
         <v>215</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="49" t="s">
-        <v>184</v>
-      </c>
-      <c r="G10" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="G10" s="22" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>217</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="12">
         <v>46260.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="12">
         <v>46261.0</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="12">
         <v>46262.0</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="11">
         <v>46264.0</v>
       </c>
     </row>
@@ -25755,36 +25775,36 @@
         <v>215</v>
       </c>
       <c r="C12" s="27"/>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="22" t="s">
         <v>220</v>
       </c>
       <c r="E12" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="F12" s="23" t="s">
+      <c r="F12" s="22" t="s">
         <v>221</v>
       </c>
       <c r="G12" s="27"/>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
     </row>
     <row r="14" ht="91.5" customHeight="1">
       <c r="A14" s="27"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -25813,84 +25833,84 @@
   <sheetData>
     <row r="1" ht="43.5" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
     <row r="2" ht="24.0" customHeight="1">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="51" t="s">
         <v>223</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8"/>
-      <c r="B3" s="21" t="s">
-        <v>224</v>
-      </c>
-      <c r="C3" s="16">
+      <c r="A3" s="9"/>
+      <c r="B3" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="C3" s="12">
         <v>46267.0</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="12">
         <v>46268.0</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="12">
         <v>46269.0</v>
       </c>
-      <c r="F3" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="G3" s="19">
+      <c r="F3" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="G3" s="11">
         <v>46271.0</v>
       </c>
     </row>
     <row r="4" ht="85.5" customHeight="1">
-      <c r="A4" s="8"/>
+      <c r="A4" s="9"/>
       <c r="B4" s="27"/>
       <c r="C4" s="27"/>
       <c r="D4" s="27"/>
-      <c r="E4" s="58" t="s">
-        <v>226</v>
+      <c r="E4" s="61" t="s">
+        <v>232</v>
       </c>
       <c r="F4" s="27"/>
       <c r="G4" s="27"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
-        <v>227</v>
-      </c>
-      <c r="B5" s="59" t="s">
-        <v>228</v>
-      </c>
-      <c r="C5" s="60">
+      <c r="A5" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="B5" s="62" t="s">
+        <v>241</v>
+      </c>
+      <c r="C5" s="64">
         <v>46274.0</v>
       </c>
-      <c r="D5" s="61">
+      <c r="D5" s="66">
         <v>46275.0</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="12">
         <v>46276.0</v>
       </c>
-      <c r="F5" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="G5" s="19">
+      <c r="F5" s="15" t="s">
+        <v>250</v>
+      </c>
+      <c r="G5" s="11">
         <v>46278.0</v>
       </c>
     </row>
     <row r="6" ht="95.25" customHeight="1">
-      <c r="A6" s="23" t="s">
-        <v>230</v>
+      <c r="A6" s="22" t="s">
+        <v>252</v>
       </c>
       <c r="B6" s="27"/>
       <c r="C6" s="27"/>
@@ -25900,37 +25920,37 @@
       <c r="G6" s="27"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
-        <v>231</v>
-      </c>
-      <c r="B7" s="59" t="s">
-        <v>232</v>
-      </c>
-      <c r="C7" s="60">
+      <c r="A7" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="B7" s="62" t="s">
+        <v>256</v>
+      </c>
+      <c r="C7" s="64">
         <v>46281.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="12">
         <v>46282.0</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="12">
         <v>46283.0</v>
       </c>
-      <c r="F7" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="G7" s="19">
+      <c r="F7" s="15" t="s">
+        <v>260</v>
+      </c>
+      <c r="G7" s="11">
         <v>46285.0</v>
       </c>
     </row>
     <row r="8" ht="94.5" customHeight="1">
-      <c r="A8" s="23" t="s">
-        <v>234</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>235</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>236</v>
+      <c r="A8" s="22" t="s">
+        <v>264</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>266</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>268</v>
       </c>
       <c r="D8" s="27"/>
       <c r="E8" s="27"/>
@@ -25938,68 +25958,68 @@
       <c r="G8" s="27"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>237</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>238</v>
-      </c>
-      <c r="C9" s="16">
+      <c r="A9" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="C9" s="12">
         <v>46288.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="12">
         <v>46289.0</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="12">
         <v>46290.0</v>
       </c>
-      <c r="F9" s="18" t="s">
-        <v>239</v>
-      </c>
-      <c r="G9" s="19">
+      <c r="F9" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="G9" s="11">
         <v>46292.0</v>
       </c>
     </row>
     <row r="10" ht="98.25" customHeight="1">
-      <c r="A10" s="63" t="s">
-        <v>241</v>
+      <c r="A10" s="69" t="s">
+        <v>278</v>
       </c>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="27"/>
-      <c r="E10" s="63" t="s">
-        <v>242</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>243</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>244</v>
+      <c r="E10" s="69" t="s">
+        <v>279</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>280</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>245</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="C11" s="16">
+      <c r="A11" s="19" t="s">
+        <v>282</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>283</v>
+      </c>
+      <c r="C11" s="12">
         <v>46295.0</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" ht="108.0" customHeight="1">
       <c r="A12" s="27"/>
       <c r="B12" s="27"/>
       <c r="C12" s="27"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>